<commit_message>
📊 Horarios actualizados Línea 141 - 2137
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:20:52</t>
+          <t>Última actualización: 02:17:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:20:52</t>
+          <t>02:17:07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:12</t>
+          <t>02:57</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,12 +498,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>00:20:52</t>
+          <t>02:17:07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01:58</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -512,9 +512,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:17:07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>03:51</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>83_ESC 6_ALUAR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>94</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:20:52</t>
+          <t>Última actualización: 02:17:07</t>
         </is>
       </c>
     </row>
@@ -585,12 +610,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:20:52</t>
+          <t>02:17:07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:12</t>
+          <t>02:57</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -599,7 +624,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -631,7 +656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:20:52</t>
+          <t>Última actualización: 02:17:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2138
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:17:07</t>
+          <t>Última actualización: 03:19:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:17:07</t>
+          <t>03:19:18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:57</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:17:07</t>
+          <t>03:19:18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>03:51</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>83_ESC 6_ALUAR</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,23 +523,98 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:17:07</t>
+          <t>03:19:18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03:51</t>
+          <t>04:32</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>83_ESC 6_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:19:18</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>89</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:19:18</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>89</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:19:18</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:07</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>108</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -569,7 +644,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:17:07</t>
+          <t>Última actualización: 03:19:18</t>
         </is>
       </c>
     </row>
@@ -610,21 +685,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:17:07</t>
+          <t>03:19:18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:57</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,7 +731,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:17:07</t>
+          <t>Última actualización: 03:19:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2139
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:19:18</t>
+          <t>Última actualización: 04:43:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:19:18</t>
+          <t>04:43:38</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:19:18</t>
+          <t>04:43:38</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:51</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>83_ESC 6_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:19:18</t>
+          <t>04:43:38</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:32</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:19:18</t>
+          <t>04:43:38</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:19:18</t>
+          <t>04:43:38</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,12 +598,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:19:18</t>
+          <t>04:43:38</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:07</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -612,9 +612,209 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>108</v>
+        <v>64</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:43:38</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>78</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:43:38</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>86</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:43:38</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>89</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:43:38</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>107</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:43:38</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>113</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:43:38</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>116</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:43:38</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>117</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>04:43:38</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>118</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -644,7 +844,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:19:18</t>
+          <t>Última actualización: 04:43:38</t>
         </is>
       </c>
     </row>
@@ -685,12 +885,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:19:18</t>
+          <t>04:43:38</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -731,7 +931,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:19:18</t>
+          <t>Última actualización: 04:43:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2140
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:43:38</t>
+          <t>Última actualización: 05:39:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>05:41</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:47</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>06:09</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:36</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>89</v>
+        <v>62</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>113</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,23 +798,73 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
+        <v>113</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>05:39:14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
         <v>118</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>05:39:14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>118</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -831,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -844,14 +894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:43:38</t>
+          <t>Última actualización: 05:39:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -885,7 +935,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:43:38</t>
+          <t>05:39:14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -899,9 +949,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>89</v>
+        <v>33</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:39:14</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>83</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:39:14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>113</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -931,7 +1031,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:43:38</t>
+          <t>Última actualización: 05:39:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2141
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:39:14</t>
+          <t>Última actualización: 06:39:39</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:41</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,12 +573,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>102</v>
+        <v>72</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>118</v>
+        <v>106</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -894,7 +894,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:39:14</t>
+          <t>Última actualización: 06:39:39</t>
         </is>
       </c>
     </row>
@@ -935,12 +935,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -960,21 +960,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -985,21 +985,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:39:14</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>113</v>
+        <v>72</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1031,14 +1031,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:39:14</t>
+          <t>Última actualización: 06:39:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:39:39</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>69</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:39:39</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>118</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2142
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:39:39</t>
+          <t>Última actualización: 07:33:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:39:39</t>
+          <t>07:33:24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:33</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -728,16 +728,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:39:39</t>
+          <t>07:33:24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:39:39</t>
+          <t>07:33:24</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:39:39</t>
+          <t>07:33:24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>100</v>
+        <v>18</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:39:39</t>
+          <t>07:33:24</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>102</v>
+        <v>28</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,23 +848,323 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>33</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>46</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>48</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>06:39:39</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>08:25</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D24" t="n">
         <v>106</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>53</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>71</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>72</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>91</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>93</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>98</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>103</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>104</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>111</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -881,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -894,14 +1194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:39:39</t>
+          <t>Última actualización: 07:33:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -985,23 +1285,123 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:39:39</t>
+          <t>07:33:24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>07:33</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>07:51</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
+        <v>18</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>71</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>72</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>93</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1018,7 +1418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1031,14 +1431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:39:39</t>
+          <t>Última actualización: 07:33:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1097,25 +1497,100 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>16</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>06:39:39</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>08:37</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D8" t="n">
         <v>118</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>65</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:33:24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2143
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:33:24</t>
+          <t>Última actualización: 08:27:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:42</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>91</v>
+        <v>18</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>93</v>
+        <v>37</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>98</v>
+        <v>39</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>103</v>
+        <v>44</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>104</v>
+        <v>49</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,23 +1148,248 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>50</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>09:24</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>111</v>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="D34" t="n">
+        <v>57</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>67</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>68</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>77</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>88</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>94</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10:06</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>99</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>108</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>117</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1181,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1194,14 +1419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:33:24</t>
+          <t>Última actualización: 08:27:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1560,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1349,7 +1574,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1360,7 +1585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1374,7 +1599,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1385,7 +1610,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1399,9 +1624,34 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>88</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1418,7 +1668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1431,14 +1681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:33:24</t>
+          <t>Última actualización: 08:27:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1522,12 +1772,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:39:39</t>
+          <t>08:27:18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>08:37</t>
+          <t>08:27</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1536,7 +1786,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1547,12 +1797,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:33:24</t>
+          <t>06:39:39</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1561,7 +1811,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1577,18 +1827,93 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>65</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>09:03</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>90</v>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D11" t="n">
+        <v>36</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>61</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>111</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2144
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:27:18</t>
+          <t>Última actualización: 09:04:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>77</v>
+        <v>31</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1278,16 +1278,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>94</v>
+        <v>47</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10:06</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>108</v>
+        <v>53</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,18 +1378,268 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>94</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>60</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>61</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>10:06</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>99</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>71</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>08:27:18</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>10:24</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D47" t="n">
         <v>117</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>81</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>100</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>100</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>111</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>113</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1419,7 +1669,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:27:18</t>
+          <t>Última actualización: 09:04:12</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1860,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1624,7 +1874,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1635,7 +1885,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1649,7 +1899,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1668,7 +1918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1681,14 +1931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:27:18</t>
+          <t>Última actualización: 09:04:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -1872,50 +2122,125 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:27:18</t>
+          <t>09:04:12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>24</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>10:18</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>111</v>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D14" t="n">
+        <v>74</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>86</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>09:04:12</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>99</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2145
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:04:12</t>
+          <t>Última actualización: 10:49:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 66</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>09:04:12</t>
+          <t>10:49:35</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>111</v>
+        <v>2</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,23 +1623,498 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>6</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>7</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>09:04:12</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>10:57</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D52" t="n">
+      <c r="D54" t="n">
         <v>113</v>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>12</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>15</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>19</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>11:16</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>27</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>35</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>46</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>47</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>51</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>55</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>65</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>66</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>75</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>86</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>95</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>105</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>107</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>115</v>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1656,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1669,14 +2144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:04:12</t>
+          <t>Última actualización: 10:49:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1902,6 +2377,56 @@
         <v>51</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>46</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>55</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1918,7 +2443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1931,14 +2456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:04:12</t>
+          <t>Última actualización: 10:49:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2241,6 +2766,31 @@
       <c r="E16" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10:49:35</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>33</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2146
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:49:35</t>
+          <t>Última actualización: 11:43:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 66</t>
+          <t>Total filas: 76</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:43</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>75</v>
+        <v>12</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>95</v>
+        <v>21</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>105</v>
+        <v>28</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>107</v>
+        <v>32</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,23 +2098,273 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>41</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>48</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>51</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>53</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
           <t>12:44</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D71" t="n">
-        <v>115</v>
-      </c>
-      <c r="E71" t="inlineStr">
+      <c r="D75" t="n">
+        <v>61</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>63</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>72</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>81</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>92</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>101</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>108</v>
+      </c>
+      <c r="E81" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2131,7 +2381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2144,14 +2394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:49:35</t>
+          <t>Última actualización: 11:43:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2660,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10:49:35</t>
+          <t>11:43:37</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2424,9 +2674,59 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>72</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>108</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2443,7 +2743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2456,14 +2756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:49:35</t>
+          <t>Última actualización: 11:43:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2789,6 +3089,31 @@
         <v>33</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>11:43:37</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>99</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2147
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:43:37</t>
+          <t>Última actualización: 12:42:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 76</t>
+          <t>Total filas: 88</t>
         </is>
       </c>
     </row>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>11:43:37</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>61</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>11:43:37</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,12 +2248,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>11:43:37</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2278,16 +2278,16 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>11:43:37</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>11:43:37</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>101</v>
+        <v>33</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,23 +2348,323 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>11:43:37</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>39</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>42</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
           <t>13:31</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D81" t="n">
-        <v>108</v>
-      </c>
-      <c r="E81" t="inlineStr">
+      <c r="D83" t="n">
+        <v>49</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>62</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>73</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>74</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>82</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>89</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>92</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>92</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>94</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>102</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>112</v>
+      </c>
+      <c r="E93" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2381,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2394,14 +2694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:43:37</t>
+          <t>Última actualización: 12:42:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2685,12 +2985,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11:43:37</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:54</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2699,7 +2999,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2715,18 +3015,68 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>72</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>13:31</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>108</v>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D18" t="n">
+        <v>49</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>112</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2743,7 +3093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2756,14 +3106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:43:37</t>
+          <t>Última actualización: 12:42:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3447,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11:43:37</t>
+          <t>12:42:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3111,11 +3461,36 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>99</v>
+        <v>40</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>67</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2148
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:42:43</t>
+          <t>Última actualización: 13:38:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 88</t>
+          <t>Total filas: 101</t>
         </is>
       </c>
     </row>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:38:04</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:38:04</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:38:04</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:38:04</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>89</v>
+        <v>26</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2553,16 +2553,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:38:04</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>92</v>
+        <v>34</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:38:04</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>94</v>
+        <v>36</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>12:42:43</t>
+          <t>13:38:04</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>102</v>
+        <v>36</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,18 +2653,343 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>94</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>39</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>102</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>47</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>12:42:43</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
           <t>14:34</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D93" t="n">
+      <c r="D97" t="n">
         <v>112</v>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>57</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>14:37</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>59</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>66</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>77</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>15:02</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>84</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>87</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>97</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>106</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>117</v>
+      </c>
+      <c r="E106" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2681,7 +3006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2694,14 +3019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:42:43</t>
+          <t>Última actualización: 13:38:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3077,6 +3402,106 @@
         <v>112</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>57</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>77</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>87</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>117</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3093,7 +3518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3106,14 +3531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:42:43</t>
+          <t>Última actualización: 13:38:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3489,6 +3914,81 @@
         <v>67</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>12</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>65</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>13:38:04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>105</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2149
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:38:04</t>
+          <t>Última actualización: 14:29:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 101</t>
+          <t>Total filas: 111</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2787,7 +2787,7 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2837,7 +2837,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>66</v>
+        <v>15</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>77</v>
+        <v>17</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>84</v>
+        <v>26</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>87</v>
+        <v>32</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2928,16 +2928,16 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>106</v>
+        <v>36</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,23 +2973,273 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>37</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>46</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>55</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D106" t="n">
-        <v>117</v>
-      </c>
-      <c r="E106" t="inlineStr">
+      <c r="D109" t="n">
+        <v>66</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>76</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>84</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>86</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>88</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>95</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>105</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>116</v>
+      </c>
+      <c r="E116" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3019,7 +3269,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:38:04</t>
+          <t>Última actualización: 14:29:13</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3660,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3424,7 +3674,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3435,7 +3685,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3449,7 +3699,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>77</v>
+        <v>26</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3460,7 +3710,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3474,7 +3724,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3485,7 +3735,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3499,7 +3749,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>117</v>
+        <v>66</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3518,7 +3768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3531,14 +3781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:38:04</t>
+          <t>Última actualización: 14:29:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3947,7 +4197,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3961,7 +4211,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>65</v>
+        <v>14</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3972,7 +4222,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>13:38:04</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3986,11 +4236,36 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>94</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2150
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E116"/>
+  <dimension ref="A1:E129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:29:13</t>
+          <t>Última actualización: 15:07:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 111</t>
+          <t>Total filas: 124</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>14:29:13</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>14:29:13</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,12 +3048,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>14:29:13</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3078,16 +3078,16 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>14:29:13</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>14:29:13</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>86</v>
+        <v>37</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3153,16 +3153,16 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>14:29:13</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>95</v>
+        <v>44</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3203,16 +3203,16 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,23 +3223,348 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>48</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>49</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
           <t>14:29:13</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>88</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>57</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>67</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>77</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
         <is>
           <t>16:25</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C122" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D116" t="n">
+      <c r="D122" t="n">
         <v>116</v>
       </c>
-      <c r="E116" t="inlineStr">
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>87</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>88</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>94</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>97</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>97</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>108</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>117</v>
+      </c>
+      <c r="E129" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3256,7 +3581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3269,14 +3594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:29:13</t>
+          <t>Última actualización: 15:07:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3735,23 +4060,48 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>27</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>14:29:13</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>15:35</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>66</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3768,7 +4118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3781,14 +4131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:29:13</t>
+          <t>Última actualización: 15:07:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4222,12 +4572,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14:29:13</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4236,7 +4586,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4252,20 +4602,95 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>54</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>55</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>14:29:13</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>16:03</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D25" t="n">
         <v>94</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>15:07:47</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>82</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2151
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:07:47</t>
+          <t>Última actualización: 16:12:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 124</t>
+          <t>Total filas: 136</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>77</v>
+        <v>12</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>14:29:13</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>116</v>
+        <v>12</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>87</v>
+        <v>12</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>14:29:13</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>97</v>
+        <v>23</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>97</v>
+        <v>29</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3528,16 +3528,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,23 +3548,323 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>32</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>39</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>43</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
           <t>15:07:47</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
+      <c r="B132" t="inlineStr">
         <is>
           <t>17:04</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
+      <c r="C132" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D129" t="n">
+      <c r="D132" t="n">
         <v>117</v>
       </c>
-      <c r="E129" t="inlineStr">
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>53</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>63</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>72</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>81</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>83</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>84</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>93</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>103</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>18:03</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>111</v>
+      </c>
+      <c r="E141" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3581,7 +3881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3594,14 +3894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:07:47</t>
+          <t>Última actualización: 16:12:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4102,6 +4402,81 @@
         <v>66</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>63</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>93</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>103</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4118,7 +4493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4131,14 +4506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:07:47</t>
+          <t>Última actualización: 16:12:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4691,6 +5066,56 @@
       <c r="E26" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>18</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>71</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2152
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E141"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:12:17</t>
+          <t>Última actualización: 16:57:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 136</t>
+          <t>Total filas: 150</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:57:45</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>117</v>
+        <v>1</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,12 +3648,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>16:57:45</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>16:57:45</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3728,16 +3728,16 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>16:57:45</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,12 +3773,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>16:57:45</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3787,7 +3787,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>16:57:45</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>103</v>
+        <v>38</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3853,18 +3853,368 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>84</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>39</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>47</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>93</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>57</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>103</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
           <t>18:03</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
+      <c r="C147" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D141" t="n">
+      <c r="D147" t="n">
         <v>111</v>
       </c>
-      <c r="E141" t="inlineStr">
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>67</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>77</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>87</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>88</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>97</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>99</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>107</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>117</v>
+      </c>
+      <c r="E155" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3881,7 +4231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3894,14 +4244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:12:17</t>
+          <t>Última actualización: 16:57:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4410,12 +4760,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>16:57:45</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4424,7 +4774,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>63</v>
+        <v>17</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4440,16 +4790,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>93</v>
+        <v>63</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4460,23 +4810,123 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>47</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>16:12:17</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>93</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>57</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>17:55</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D30" t="n">
         <v>103</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>77</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4493,7 +4943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4506,14 +4956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:12:17</t>
+          <t>Última actualización: 16:57:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5097,23 +5547,73 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>25</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>16:12:17</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D29" t="n">
         <v>71</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>16:57:45</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>107</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2153
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:57:45</t>
+          <t>Última actualización: 17:30:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 150</t>
+          <t>Total filas: 159</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3853,16 +3853,16 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3928,16 +3928,16 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3978,16 +3978,16 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>18:03</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>111</v>
+        <v>24</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>87</v>
+        <v>34</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4128,16 +4128,16 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4153,16 +4153,16 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:29</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,23 +4198,248 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>64</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>66</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>74</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
           <t>18:54</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C158" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D155" t="n">
-        <v>117</v>
-      </c>
-      <c r="E155" t="inlineStr">
+      <c r="D158" t="n">
+        <v>84</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>18:57</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>87</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>89</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>94</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>106</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>114</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>114</v>
+      </c>
+      <c r="E164" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4231,7 +4456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4244,14 +4469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:57:45</t>
+          <t>Última actualización: 17:30:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -4810,21 +5035,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4835,12 +5060,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4849,7 +5074,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>93</v>
+        <v>14</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4860,21 +5085,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -4885,12 +5110,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4899,7 +5124,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>103</v>
+        <v>24</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -4910,23 +5135,98 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>16:12:17</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>103</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>16:57:45</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>18:14</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D32" t="n">
         <v>77</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>89</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>114</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4943,7 +5243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4956,14 +5256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:57:45</t>
+          <t>Última actualización: 17:30:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -5616,6 +5916,56 @@
       <c r="E30" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>83</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>19:14</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>104</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2154
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:30:45</t>
+          <t>Última actualización: 18:05:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 159</t>
+          <t>Total filas: 170</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>84</v>
+        <v>6</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>16:57:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4153,16 +4153,16 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>18:29</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>16:57:45</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>16:57:45</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4278,16 +4278,16 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:29</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>18:57</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>87</v>
+        <v>29</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>18:59</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>106</v>
+        <v>49</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4403,16 +4403,16 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>18:57</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4428,18 +4428,293 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>89</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>55</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>59</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>71</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>106</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>74</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
           <t>19:24</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>79</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D164" t="n">
+      <c r="D171" t="n">
         <v>114</v>
       </c>
-      <c r="E164" t="inlineStr">
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>80</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>19:26</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>81</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>104</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>105</v>
+      </c>
+      <c r="E175" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4456,7 +4731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4469,14 +4744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:30:45</t>
+          <t>Última actualización: 18:05:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -5185,21 +5460,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>18:59</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5215,18 +5490,93 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>18:59</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>89</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>55</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>17:30:45</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>19:24</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D36" t="n">
         <v>114</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>80</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5243,7 +5593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5256,14 +5606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:30:45</t>
+          <t>Última actualización: 18:05:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -5966,6 +6316,81 @@
       <c r="E32" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>70</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>83</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>102</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2155
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:05:32</t>
+          <t>Última actualización: 18:49:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 170</t>
+          <t>Total filas: 179</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>84</v>
+        <v>6</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4423,7 +4423,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,12 +4498,12 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>106</v>
+        <v>27</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4553,16 +4553,16 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>104</v>
+        <v>35</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4703,18 +4703,243 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>80</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>18:05:32</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>19:26</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>81</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>60</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C178" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D175" t="n">
-        <v>105</v>
-      </c>
-      <c r="E175" t="inlineStr">
+      <c r="D178" t="n">
+        <v>61</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>20:08</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>79</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>85</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>86</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>107</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>110</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>113</v>
+      </c>
+      <c r="E184" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4731,7 +4956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4744,14 +4969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:05:32</t>
+          <t>Última actualización: 18:49:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5710,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5499,7 +5724,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5535,7 +5760,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5549,7 +5774,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>114</v>
+        <v>35</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5577,6 +5802,56 @@
         <v>80</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>85</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>110</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5593,7 +5868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5606,14 +5881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:05:32</t>
+          <t>Última actualización: 18:49:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6572,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6311,7 +6586,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6372,23 +6647,73 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>57</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>18:05:32</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>19:47</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D36" t="n">
         <v>102</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>112</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2156
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E184"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:49:40</t>
+          <t>Última actualización: 19:19:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 179</t>
+          <t>Total filas: 189</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4558,11 +4558,11 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4653,16 +4653,16 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>81</v>
+        <v>6</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>20:08</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>85</v>
+        <v>31</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>86</v>
+        <v>37</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4878,16 +4878,16 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:08</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>107</v>
+        <v>79</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>110</v>
+        <v>53</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4928,18 +4928,268 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>85</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>86</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>56</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>57</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>77</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>18:49:40</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>110</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>81</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
           <t>20:42</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr">
+      <c r="C191" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D184" t="n">
-        <v>113</v>
-      </c>
-      <c r="E184" t="inlineStr">
+      <c r="D191" t="n">
+        <v>83</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>92</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>98</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>108</v>
+      </c>
+      <c r="E194" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4956,7 +5206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4969,14 +5219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:49:40</t>
+          <t>Última actualización: 19:19:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -5785,7 +6035,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -5799,7 +6049,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>80</v>
+        <v>6</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -5835,23 +6085,73 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>56</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>18:49:40</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>20:39</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D40" t="n">
         <v>110</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>81</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5868,7 +6168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5881,14 +6181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:49:40</t>
+          <t>Última actualización: 19:19:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6972,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6686,7 +6986,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>102</v>
+        <v>28</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6697,23 +6997,48 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>19:19:13</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>80</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>18:49:40</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D38" t="n">
         <v>112</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2157
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:19:13</t>
+          <t>Última actualización: 19:53:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 189</t>
+          <t>Total filas: 195</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>84</v>
+        <v>6</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4558,11 +4558,11 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>27</v>
+        <v>106</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>106</v>
+        <v>27</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,12 +4873,12 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>20:08</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>79</v>
+        <v>8</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,12 +4898,12 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>20:12</t>
+          <t>20:08</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4953,16 +4953,16 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>57</v>
+        <v>22</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>110</v>
+        <v>43</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,12 +5073,12 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5103,16 +5103,16 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>92</v>
+        <v>49</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5153,16 +5153,16 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,23 +5173,173 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
+          <t>19:53:33</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>62</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>19:53:33</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>63</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
           <t>19:19:13</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr">
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>98</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>19:53:33</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>72</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>19:53:33</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
         <is>
           <t>21:07</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
+      <c r="C198" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D194" t="n">
-        <v>108</v>
-      </c>
-      <c r="E194" t="inlineStr">
+      <c r="D198" t="n">
+        <v>74</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>19:53:33</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>101</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>19:53:33</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>104</v>
+      </c>
+      <c r="E200" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5219,7 +5369,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:19:13</t>
+          <t>Última actualización: 19:53:33</t>
         </is>
       </c>
     </row>
@@ -6085,7 +6235,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6099,7 +6249,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6110,7 +6260,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6124,7 +6274,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>110</v>
+        <v>46</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6168,7 +6318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6181,14 +6331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:19:13</t>
+          <t>Última actualización: 19:53:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -7039,6 +7189,56 @@
         <v>112</v>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>19:53:33</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>68</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>19:53:33</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>99</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2158
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E200"/>
+  <dimension ref="A1:E205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:53:33</t>
+          <t>Última actualización: 20:23:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 195</t>
+          <t>Total filas: 200</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>84</v>
+        <v>6</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>19:53:33</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>22</v>
+        <v>86</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>19:53:33</t>
+          <t>20:23:06</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>20:23:06</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>19:53:33</t>
+          <t>20:23:06</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5173,12 +5173,12 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>19:53:33</t>
+          <t>20:23:06</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5203,16 +5203,16 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,12 +5223,12 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>19:53:33</t>
+          <t>20:23:06</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>72</v>
+        <v>34</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5278,16 +5278,16 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>21:07</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>19:53:33</t>
+          <t>20:23:06</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>101</v>
+        <v>43</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,23 +5323,148 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>19:53:33</t>
+          <t>20:23:06</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>44</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>20:23:06</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>71</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>20:23:06</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>73</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>20:23:06</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
           <t>21:37</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr">
+      <c r="C203" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D200" t="n">
-        <v>104</v>
-      </c>
-      <c r="E200" t="inlineStr">
+      <c r="D203" t="n">
+        <v>74</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>20:23:06</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>77</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>20:23:06</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>96</v>
+      </c>
+      <c r="E205" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5369,7 +5494,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:53:33</t>
+          <t>Última actualización: 20:23:06</t>
         </is>
       </c>
     </row>
@@ -6285,7 +6410,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>20:23:06</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -6299,7 +6424,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -6318,7 +6443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6331,14 +6456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:53:33</t>
+          <t>Última actualización: 20:23:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -7197,12 +7322,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>19:53:33</t>
+          <t>20:23:06</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -7211,7 +7336,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7227,20 +7352,70 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>68</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>20:23:06</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>21:32</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>99</v>
-      </c>
-      <c r="E40" t="inlineStr">
+      <c r="D41" t="n">
+        <v>69</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20:23:06</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>106</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2159
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E205"/>
+  <dimension ref="A1:E209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:23:06</t>
+          <t>Última actualización: 20:55:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 200</t>
+          <t>Total filas: 204</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D123" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>84</v>
+        <v>6</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4558,11 +4558,11 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>27</v>
+        <v>106</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>20:23:06</t>
+          <t>20:55:04</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>20:23:06</t>
+          <t>20:55:04</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5312,7 +5312,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>20:23:06</t>
+          <t>20:55:04</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>20:23:06</t>
+          <t>20:55:04</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>20:23:06</t>
+          <t>20:55:04</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>73</v>
+        <v>41</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>20:23:06</t>
+          <t>20:55:04</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>20:23:06</t>
+          <t>20:55:04</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>77</v>
+        <v>45</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>20:23:06</t>
+          <t>20:55:04</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5462,9 +5462,109 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>96</v>
+        <v>64</v>
       </c>
       <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>20:55:04</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>72</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>20:55:04</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>91</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>20:55:04</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>102</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>20:55:04</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>106</v>
+      </c>
+      <c r="E209" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5481,7 +5581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5494,14 +5594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:23:06</t>
+          <t>Última actualización: 20:55:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -6427,6 +6527,31 @@
         <v>17</v>
       </c>
       <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>20:55:04</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>102</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6443,7 +6568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6456,14 +6581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:23:06</t>
+          <t>Última actualización: 20:55:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -7372,12 +7497,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>20:23:06</t>
+          <t>20:55:04</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>21:32</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -7386,7 +7511,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>69</v>
+        <v>10</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7402,18 +7527,68 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>69</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>20:55:04</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>40</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>20:55:04</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>22:09</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D42" t="n">
-        <v>106</v>
-      </c>
-      <c r="E42" t="inlineStr">
+      <c r="D44" t="n">
+        <v>74</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2160
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-02.xlsx
+++ b/data/horarios-141-2026-04-02.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E209"/>
+  <dimension ref="A1:E216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:55:04</t>
+          <t>Última actualización: 22:14:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 204</t>
+          <t>Total filas: 211</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>15:07:47</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>15:07:47</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>32</v>
+        <v>97</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D138" t="n">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D139" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>16:12:17</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>84</v>
+        <v>6</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>16:12:17</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>6</v>
+        <v>84</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>17:30:45</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4558,11 +4558,11 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>17:30:45</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>18:05:32</t>
+          <t>19:19:13</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>19:19:13</t>
+          <t>18:05:32</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4633,11 +4633,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>19:53:33</t>
+          <t>18:49:40</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>22</v>
+        <v>86</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>18:49:40</t>
+          <t>19:53:33</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>20:55:04</t>
+          <t>22:14:11</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>91</v>
+        <v>12</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>20:55:04</t>
+          <t>22:14:11</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>22:37</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>102</v>
+        <v>21</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,23 +5548,198 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
+          <t>22:14:11</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>23</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
           <t>20:55:04</t>
         </is>
       </c>
-      <c r="B209" t="inlineStr">
+      <c r="B210" t="inlineStr">
         <is>
           <t>22:41</t>
         </is>
       </c>
-      <c r="C209" t="inlineStr">
+      <c r="C210" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D209" t="n">
+      <c r="D210" t="n">
         <v>106</v>
       </c>
-      <c r="E209" t="inlineStr">
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>22:14:11</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>22:48</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>34</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>22:14:11</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>22:56</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>42</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>22:14:11</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>23:07</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>53</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>22:14:11</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>23:26</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>72</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>22:14:11</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>23:41</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>87</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>22:14:11</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>23:55</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>101</v>
+      </c>
+      <c r="E216" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5581,7 +5756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5594,14 +5769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:55:04</t>
+          <t>Última actualización: 22:14:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -6535,7 +6710,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>20:55:04</t>
+          <t>22:14:11</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -6549,9 +6724,34 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>102</v>
+        <v>23</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>22:14:11</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>23:41</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>87</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6581,7 +6781,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:55:04</t>
+          <t>Última actualización: 22:14:11</t>
         </is>
       </c>
     </row>

</xml_diff>